<commit_message>
add: topic - arrays - P06_left_rotate_array_by_one
</commit_message>
<xml_diff>
--- a/topics/leetcode.xlsx
+++ b/topics/leetcode.xlsx
@@ -16,18 +16,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <r>
-      <rPr>
-        <b val="false"/>
-        <i val="false"/>
-        <sz val="20"/>
-        <color indexed="2"/>
-        <rFont val="Arial Black"/>
-      </rPr>
-      <t>PROBLEMS</t>
-    </r>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>PROBLEMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repository -</t>
+  </si>
+  <si>
+    <t>Link</t>
   </si>
   <si>
     <r>
@@ -123,6 +123,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Largest Element</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="false"/>
@@ -134,6 +137,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Second Largest Element</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="false"/>
@@ -145,6 +151,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Second Smallest Element</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="false"/>
@@ -156,6 +165,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Array is Sorted</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="false"/>
@@ -183,29 +195,23 @@
         <b val="false"/>
         <i val="false"/>
         <sz val="11"/>
-        <color indexed="4"/>
-        <rFont val="Liberation Sans"/>
-      </rPr>
-      <t>Link</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="false"/>
-        <i val="false"/>
-        <sz val="11"/>
         <rFont val="Liberation Sans"/>
       </rPr>
       <t>Completed</t>
     </r>
+  </si>
+  <si>
+    <t>P06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Left Rotate Array by One</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -213,11 +219,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="0"/>
+      <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
       <i val="0"/>
       <sz val="20.000000"/>
       <color indexed="2"/>
-      <name val="Arial Black"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -236,14 +259,6 @@
       <b/>
       <i val="0"/>
       <sz val="11.000000"/>
-      <name val="Liberation Sans"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <u/>
-      <sz val="11.000000"/>
-      <color indexed="4"/>
       <name val="Liberation Sans"/>
     </font>
   </fonts>
@@ -274,7 +289,7 @@
       <right style="none"/>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -295,16 +310,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -312,43 +327,81 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="5" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="5" fillId="2" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -849,188 +902,716 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="4" width="10.682"/>
-    <col customWidth="1" min="5" max="5" width="47.003900000000002"/>
-    <col customWidth="1" min="6" max="8" width="15.0039"/>
+    <col customWidth="1" min="1" max="1" style="1" width="4.28125"/>
+    <col customWidth="1" min="2" max="2" style="2" width="14.00390625"/>
+    <col customWidth="1" min="3" max="3" style="2" width="16.421875"/>
+    <col customWidth="1" min="4" max="4" style="1" width="10.682"/>
+    <col customWidth="1" min="5" max="5" style="3" width="47.003900000000002"/>
+    <col customWidth="1" min="6" max="8" style="4" width="15.0039"/>
+    <col min="9" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" ht="14.25">
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" ht="30">
-      <c r="B3" s="2" t="s">
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" ht="24">
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" ht="14.25">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" ht="14.25">
-      <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" ht="28.5">
-      <c r="B6" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="7" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="B6" s="12"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" ht="28.5">
+      <c r="B7" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="16"/>
+      <c r="F7" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="20"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" ht="14.25">
-      <c r="B7" s="1"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" ht="14.25">
-      <c r="B8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" ht="14.25">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
     </row>
     <row r="10" ht="14.25">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="20"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="20" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="20" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>14</v>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="20"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="20" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="20"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="20" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="E36" s="3"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" ht="14.25">
+      <c r="E42" s="3"/>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="E43" s="3"/>
+    </row>
+    <row r="44" ht="14.25">
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="E45" s="3"/>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="E46" s="3"/>
+    </row>
+    <row r="47" ht="14.25">
+      <c r="E47" s="3"/>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="E48" s="3"/>
+    </row>
+    <row r="49" ht="14.25">
+      <c r="E49" s="3"/>
+    </row>
+    <row r="50" ht="14.25">
+      <c r="E50" s="3"/>
+    </row>
+    <row r="51" ht="14.25">
+      <c r="E51" s="3"/>
+    </row>
+    <row r="52" ht="14.25">
+      <c r="E52" s="3"/>
+    </row>
+    <row r="53" ht="14.25">
+      <c r="E53" s="3"/>
+    </row>
+    <row r="54" ht="14.25">
+      <c r="E54" s="3"/>
+    </row>
+    <row r="55" ht="14.25">
+      <c r="E55" s="3"/>
+    </row>
+    <row r="56" ht="14.25">
+      <c r="E56" s="3"/>
+    </row>
+    <row r="57" ht="14.25">
+      <c r="E57" s="3"/>
+    </row>
+    <row r="58" ht="14.25">
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" ht="14.25">
+      <c r="E59" s="3"/>
+    </row>
+    <row r="60" ht="14.25">
+      <c r="E60" s="3"/>
+    </row>
+    <row r="61" ht="14.25">
+      <c r="E61" s="3"/>
+    </row>
+    <row r="62" ht="14.25">
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" ht="14.25">
+      <c r="E65" s="3"/>
+    </row>
+    <row r="66" ht="14.25">
+      <c r="E66" s="3"/>
+    </row>
+    <row r="67" ht="14.25">
+      <c r="E67" s="3"/>
+    </row>
+    <row r="68" ht="14.25">
+      <c r="E68" s="3"/>
+    </row>
+    <row r="69" ht="14.25">
+      <c r="E69" s="3"/>
+    </row>
+    <row r="70" ht="14.25">
+      <c r="E70" s="3"/>
+    </row>
+    <row r="71" ht="14.25">
+      <c r="E71" s="3"/>
+    </row>
+    <row r="72" ht="14.25">
+      <c r="E72" s="3"/>
+    </row>
+    <row r="73" ht="14.25">
+      <c r="E73" s="3"/>
+    </row>
+    <row r="74" ht="14.25">
+      <c r="E74" s="3"/>
+    </row>
+    <row r="75" ht="14.25">
+      <c r="E75" s="3"/>
+    </row>
+    <row r="76" ht="14.25">
+      <c r="E76" s="3"/>
+    </row>
+    <row r="77" ht="14.25">
+      <c r="E77" s="3"/>
+    </row>
+    <row r="78" ht="14.25">
+      <c r="E78" s="3"/>
+    </row>
+    <row r="79" ht="14.25">
+      <c r="E79" s="3"/>
+    </row>
+    <row r="80" ht="14.25">
+      <c r="E80" s="3"/>
+    </row>
+    <row r="81" ht="14.25">
+      <c r="E81" s="3"/>
+    </row>
+    <row r="82" ht="14.25">
+      <c r="E82" s="3"/>
+    </row>
+    <row r="83" ht="14.25">
+      <c r="E83" s="3"/>
+    </row>
+    <row r="84" ht="14.25">
+      <c r="E84" s="3"/>
+    </row>
+    <row r="85" ht="14.25">
+      <c r="E85" s="3"/>
+    </row>
+    <row r="86" ht="14.25">
+      <c r="E86" s="3"/>
+    </row>
+    <row r="87" ht="14.25">
+      <c r="E87" s="3"/>
+    </row>
+    <row r="88" ht="14.25">
+      <c r="E88" s="3"/>
+    </row>
+    <row r="89" ht="14.25">
+      <c r="E89" s="3"/>
+    </row>
+    <row r="90" ht="14.25">
+      <c r="E90" s="3"/>
+    </row>
+    <row r="91" ht="14.25">
+      <c r="E91" s="3"/>
+    </row>
+    <row r="92" ht="14.25">
+      <c r="E92" s="3"/>
+    </row>
+    <row r="93" ht="14.25">
+      <c r="E93" s="3"/>
+    </row>
+    <row r="94" ht="14.25">
+      <c r="E94" s="3"/>
+    </row>
+    <row r="95" ht="14.25">
+      <c r="E95" s="3"/>
+    </row>
+    <row r="96" ht="14.25">
+      <c r="E96" s="3"/>
+    </row>
+    <row r="97" ht="14.25">
+      <c r="E97" s="3"/>
+    </row>
+    <row r="98" ht="14.25">
+      <c r="E98" s="3"/>
+    </row>
+    <row r="99" ht="14.25">
+      <c r="E99" s="3"/>
+    </row>
+    <row r="100" ht="14.25">
+      <c r="E100" s="3"/>
+    </row>
+    <row r="101" ht="14.25">
+      <c r="E101" s="3"/>
+    </row>
+    <row r="102" ht="14.25">
+      <c r="E102" s="3"/>
+    </row>
+    <row r="103" ht="14.25">
+      <c r="E103" s="3"/>
+    </row>
+    <row r="104" ht="14.25">
+      <c r="E104" s="3"/>
+    </row>
+    <row r="105" ht="14.25">
+      <c r="E105" s="3"/>
+    </row>
+    <row r="106" ht="14.25">
+      <c r="E106" s="3"/>
+    </row>
+    <row r="107" ht="14.25">
+      <c r="E107" s="3"/>
+    </row>
+    <row r="108" ht="14.25">
+      <c r="E108" s="3"/>
+    </row>
+    <row r="109" ht="14.25">
+      <c r="E109" s="3"/>
+    </row>
+    <row r="110" ht="14.25">
+      <c r="E110" s="3"/>
+    </row>
+    <row r="111" ht="14.25">
+      <c r="E111" s="3"/>
+    </row>
+    <row r="112" ht="14.25">
+      <c r="E112" s="3"/>
+    </row>
+    <row r="113" ht="14.25">
+      <c r="E113" s="3"/>
+    </row>
+    <row r="114" ht="14.25">
+      <c r="E114" s="3"/>
+    </row>
+    <row r="115" ht="14.25">
+      <c r="E115" s="3"/>
+    </row>
+    <row r="116" ht="14.25">
+      <c r="E116" s="3"/>
+    </row>
+    <row r="117" ht="14.25">
+      <c r="E117" s="3"/>
+    </row>
+    <row r="118" ht="14.25">
+      <c r="E118" s="3"/>
+    </row>
+    <row r="119" ht="14.25">
+      <c r="E119" s="3"/>
+    </row>
+    <row r="120" ht="14.25">
+      <c r="E120" s="3"/>
+    </row>
+    <row r="121" ht="14.25">
+      <c r="E121" s="3"/>
+    </row>
+    <row r="122" ht="14.25">
+      <c r="E122" s="3"/>
+    </row>
+    <row r="123" ht="14.25">
+      <c r="E123" s="3"/>
+    </row>
+    <row r="124" ht="14.25">
+      <c r="E124" s="3"/>
+    </row>
+    <row r="125" ht="14.25">
+      <c r="E125" s="3"/>
+    </row>
+    <row r="126" ht="14.25">
+      <c r="E126" s="3"/>
+    </row>
+    <row r="127" ht="14.25">
+      <c r="E127" s="3"/>
+    </row>
+    <row r="128" ht="14.25">
+      <c r="E128" s="3"/>
+    </row>
+    <row r="129" ht="14.25">
+      <c r="E129" s="3"/>
+    </row>
+    <row r="130" ht="14.25">
+      <c r="E130" s="3"/>
+    </row>
+    <row r="131" ht="14.25">
+      <c r="E131" s="3"/>
+    </row>
+    <row r="132" ht="14.25">
+      <c r="E132" s="3"/>
+    </row>
+    <row r="133" ht="14.25">
+      <c r="E133" s="3"/>
+    </row>
+    <row r="134" ht="14.25">
+      <c r="E134" s="3"/>
+    </row>
+    <row r="135" ht="14.25">
+      <c r="E135" s="3"/>
+    </row>
+    <row r="136" ht="14.25">
+      <c r="E136" s="3"/>
+    </row>
+    <row r="137" ht="14.25">
+      <c r="E137" s="3"/>
+    </row>
+    <row r="138" ht="14.25">
+      <c r="E138" s="3"/>
+    </row>
+    <row r="139" ht="14.25">
+      <c r="E139" s="3"/>
+    </row>
+    <row r="140" ht="14.25">
+      <c r="E140" s="3"/>
+    </row>
+    <row r="141" ht="14.25">
+      <c r="E141" s="3"/>
+    </row>
+    <row r="142" ht="14.25">
+      <c r="E142" s="3"/>
+    </row>
+    <row r="143" ht="14.25">
+      <c r="E143" s="3"/>
+    </row>
+    <row r="144" ht="14.25">
+      <c r="E144" s="3"/>
+    </row>
+    <row r="145" ht="14.25">
+      <c r="E145" s="3"/>
+    </row>
+    <row r="146" ht="14.25">
+      <c r="E146" s="3"/>
+    </row>
+    <row r="147" ht="14.25">
+      <c r="E147" s="3"/>
+    </row>
+    <row r="148" ht="14.25">
+      <c r="E148" s="3"/>
+    </row>
+    <row r="149" ht="14.25">
+      <c r="E149" s="3"/>
+    </row>
+    <row r="150" ht="14.25">
+      <c r="E150" s="3"/>
+    </row>
+    <row r="151" ht="14.25">
+      <c r="E151" s="3"/>
+    </row>
+    <row r="152" ht="14.25">
+      <c r="E152" s="3"/>
+    </row>
+    <row r="153" ht="14.25">
+      <c r="E153" s="3"/>
+    </row>
+    <row r="154" ht="14.25">
+      <c r="E154" s="3"/>
+    </row>
+    <row r="155" ht="14.25">
+      <c r="E155" s="3"/>
+    </row>
+    <row r="156" ht="14.25">
+      <c r="E156" s="3"/>
+    </row>
+    <row r="157" ht="14.25">
+      <c r="E157" s="3"/>
+    </row>
+    <row r="158" ht="14.25">
+      <c r="E158" s="3"/>
+    </row>
+    <row r="159" ht="14.25">
+      <c r="E159" s="3"/>
+    </row>
+    <row r="160" ht="14.25">
+      <c r="E160" s="3"/>
+    </row>
+    <row r="161" ht="14.25">
+      <c r="E161" s="3"/>
+    </row>
+    <row r="162" ht="14.25">
+      <c r="E162" s="3"/>
+    </row>
+    <row r="163" ht="14.25">
+      <c r="E163" s="3"/>
+    </row>
+    <row r="164" ht="14.25">
+      <c r="E164" s="3"/>
+    </row>
+    <row r="165" ht="14.25">
+      <c r="E165" s="3"/>
+    </row>
+    <row r="166" ht="14.25">
+      <c r="E166" s="3"/>
+    </row>
+    <row r="167" ht="14.25">
+      <c r="E167" s="3"/>
+    </row>
+    <row r="168" ht="14.25">
+      <c r="E168" s="3"/>
+    </row>
+    <row r="169" ht="14.25">
+      <c r="E169" s="3"/>
+    </row>
+    <row r="170" ht="14.25">
+      <c r="E170" s="3"/>
+    </row>
+    <row r="171" ht="14.25">
+      <c r="E171" s="3"/>
+    </row>
+    <row r="172" ht="14.25">
+      <c r="E172" s="3"/>
+    </row>
+    <row r="173" ht="14.25">
+      <c r="E173" s="3"/>
+    </row>
+    <row r="174" ht="14.25">
+      <c r="E174" s="3"/>
+    </row>
+    <row r="175" ht="14.25">
+      <c r="E175" s="3"/>
+    </row>
+    <row r="176" ht="14.25">
+      <c r="E176" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F12"/>
-    <hyperlink r:id="rId2" ref="H12"/>
+    <hyperlink r:id="rId1" ref="C4" tooltip=""/>
+    <hyperlink r:id="rId2" ref="H9" tooltip=""/>
+    <hyperlink r:id="rId3" ref="H10" tooltip=""/>
+    <hyperlink r:id="rId4" ref="H11" tooltip=""/>
+    <hyperlink r:id="rId5" ref="H12" tooltip=""/>
+    <hyperlink r:id="rId6" ref="F13"/>
+    <hyperlink r:id="rId7" ref="H13"/>
+    <hyperlink r:id="rId8" ref="H14" tooltip=""/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>